<commit_message>
Generar boletines para varios cursos
Permite seleccionar uno, varios o todos los cursos y reutiliza el pipeline existente para crear un libro independiente por curso.

Mantiene sin cambios la generación individual y por curso, y agrega cobertura para la nueva operación.

Closes #20
</commit_message>
<xml_diff>
--- a/src/Generador_EPS.xlsx
+++ b/src/Generador_EPS.xlsx
@@ -14946,7 +14946,7 @@
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>1º bimestre + 1º cuatrimestre + 3º bimestre · generación individual y por curso</x:v>
+        <x:v>1º bimestre + 1º cuatrimestre + 3º bimestre · generación individual, por curso y de varios cursos</x:v>
       </x:c>
       <x:c r="B2" s="102" t="str"/>
       <x:c r="C2" s="102" t="str"/>
@@ -15094,75 +15094,69 @@
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
       <x:c r="A14" s="82" t="str">
-        <x:v>Manual breve</x:v>
+        <x:v>Varios cursos</x:v>
       </x:c>
-      <x:c r="B14" s="82" t="str"/>
-      <x:c r="C14" s="82" t="str"/>
+      <x:c r="B14" s="82" t="str">
+        <x:v>Generar</x:v>
+      </x:c>
+      <x:c r="C14" s="82" t="str">
+        <x:v>Observaciones</x:v>
+      </x:c>
       <x:c r="D14" s="102" t="str"/>
-      <x:c r="E14" s="82" t="str">
-        <x:v>Valores válidos</x:v>
-      </x:c>
-      <x:c r="F14" s="82" t="str"/>
+      <x:c r="E14" s="102" t="str"/>
+      <x:c r="F14" s="102" t="str"/>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
-      <x:c r="A15" s="102" t="str">
-        <x:v>1. Elegir período: 1º bimestre, 1º cuatrimestre o 3º bimestre.</x:v>
+      <x:c r="A15" s="90" t="str">
+        <x:v>Informática 1 (EPSI EPS1)</x:v>
       </x:c>
       <x:c r="B15" s="102" t="str"/>
-      <x:c r="C15" s="102" t="str"/>
+      <x:c r="C15" s="102" t="str">
+        <x:v>SÍ incluye el curso en Informes EPS &gt; Generar boletines de los cursos marcados.</x:v>
+      </x:c>
       <x:c r="D15" s="102" t="str"/>
-      <x:c r="E15" s="102" t="str">
-        <x:v>1º y 3º bimestre</x:v>
-      </x:c>
-      <x:c r="F15" s="102" t="str">
-        <x:v>En proceso; Suficiente; Avanzado; ACREDITÓ</x:v>
-      </x:c>
+      <x:c r="E15" s="102" t="str"/>
+      <x:c r="F15" s="102" t="str"/>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
-      <x:c r="A16" s="102" t="str">
-        <x:v>2. Elegir hoja origen: EPSI o EPSG.</x:v>
+      <x:c r="A16" s="90" t="str">
+        <x:v>Informática 2 (EPSI EPS2)</x:v>
       </x:c>
       <x:c r="B16" s="102" t="str"/>
-      <x:c r="C16" s="102" t="str"/>
+      <x:c r="C16" s="102" t="str">
+        <x:v>Informes EPS &gt; Generar boletines de todos los cursos genera los 8 sin mirar estas marcas.</x:v>
+      </x:c>
       <x:c r="D16" s="102" t="str"/>
-      <x:c r="E16" s="102" t="str">
-        <x:v>1º cuatrimestre</x:v>
-      </x:c>
-      <x:c r="F16" s="102" t="str">
-        <x:v>Enteros 1 a 10; ACREDITÓ</x:v>
-      </x:c>
+      <x:c r="E16" s="102" t="str"/>
+      <x:c r="F16" s="102" t="str"/>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
-      <x:c r="A17" s="102" t="str">
-        <x:v>3. Ingresar DNI y verificar las URL/ID de fuentes.</x:v>
+      <x:c r="A17" s="90" t="str">
+        <x:v>Informática 3 (EPSI EPS3)</x:v>
       </x:c>
       <x:c r="B17" s="102" t="str"/>
-      <x:c r="C17" s="102" t="str"/>
+      <x:c r="C17" s="102" t="str">
+        <x:v>Usan el período, el ciclo lectivo y las fuentes de arriba; ignoran hoja origen, DNI y nivel.</x:v>
+      </x:c>
       <x:c r="D17" s="102" t="str"/>
-      <x:c r="E17" s="102" t="str">
-        <x:v>Excluidos</x:v>
-      </x:c>
-      <x:c r="F17" s="102" t="str">
-        <x:v>vacío; NO CURSA; CURSA</x:v>
-      </x:c>
+      <x:c r="E17" s="102" t="str"/>
+      <x:c r="F17" s="102" t="str"/>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
-      <x:c r="A18" s="102" t="str">
-        <x:v>4. Ejecutar Informes EPS &gt; Generar informe actual.</x:v>
+      <x:c r="A18" s="90" t="str">
+        <x:v>Informática 4 (EPSI EPS4)</x:v>
       </x:c>
       <x:c r="B18" s="102" t="str"/>
-      <x:c r="C18" s="102" t="str"/>
+      <x:c r="C18" s="102" t="str">
+        <x:v>Un libro por curso, como la generación por curso. Un curso sin estudiantes listos no genera libro.</x:v>
+      </x:c>
       <x:c r="D18" s="102" t="str"/>
-      <x:c r="E18" s="102" t="str">
-        <x:v>No válidos 1º cuat.</x:v>
-      </x:c>
-      <x:c r="F18" s="102" t="str">
-        <x:v>decimales; texto junto con número; nota escrita como texto</x:v>
-      </x:c>
+      <x:c r="E18" s="102" t="str"/>
+      <x:c r="F18" s="102" t="str"/>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
-      <x:c r="A19" s="102" t="str">
-        <x:v>5. Revisar Informe_actual antes de imprimir o exportar.</x:v>
+      <x:c r="A19" s="90" t="str">
+        <x:v>Gastronomía 1 (EPSG EPS1)</x:v>
       </x:c>
       <x:c r="B19" s="102" t="str"/>
       <x:c r="C19" s="102" t="str"/>
@@ -15171,65 +15165,181 @@
       <x:c r="F19" s="102" t="str"/>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
-      <x:c r="A20" s="102" t="str"/>
+      <x:c r="A20" s="90" t="str">
+        <x:v>Gastronomía 2 (EPSG EPS2)</x:v>
+      </x:c>
       <x:c r="B20" s="102" t="str"/>
       <x:c r="C20" s="102" t="str"/>
       <x:c r="D20" s="102" t="str"/>
       <x:c r="E20" s="102" t="str"/>
       <x:c r="F20" s="102" t="str"/>
     </x:row>
-    <x:row r="21" ht="30" customHeight="1">
-      <x:c r="A21" s="82" t="str">
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" s="90" t="str">
+        <x:v>Gastronomía 3 (EPSG EPS3)</x:v>
+      </x:c>
+      <x:c r="B21" s="102" t="str"/>
+      <x:c r="C21" s="102" t="str"/>
+      <x:c r="D21" s="102" t="str"/>
+      <x:c r="E21" s="102" t="str"/>
+      <x:c r="F21" s="102" t="str"/>
+    </x:row>
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="A22" s="90" t="str">
+        <x:v>Gastronomía 4 (EPSG EPS4)</x:v>
+      </x:c>
+      <x:c r="B22" s="102" t="str"/>
+      <x:c r="C22" s="102" t="str"/>
+      <x:c r="D22" s="102" t="str"/>
+      <x:c r="E22" s="102" t="str"/>
+      <x:c r="F22" s="102" t="str"/>
+    </x:row>
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="A23" s="102" t="str"/>
+      <x:c r="B23" s="102" t="str"/>
+      <x:c r="C23" s="102" t="str"/>
+      <x:c r="D23" s="102" t="str"/>
+      <x:c r="E23" s="102" t="str"/>
+      <x:c r="F23" s="102" t="str"/>
+    </x:row>
+    <x:row r="24" ht="30" customHeight="1">
+      <x:c r="A24" s="82" t="str">
+        <x:v>Manual breve</x:v>
+      </x:c>
+      <x:c r="B24" s="82" t="str"/>
+      <x:c r="C24" s="82" t="str"/>
+      <x:c r="D24" s="102" t="str"/>
+      <x:c r="E24" s="82" t="str">
+        <x:v>Valores válidos</x:v>
+      </x:c>
+      <x:c r="F24" s="82" t="str"/>
+    </x:row>
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="A25" s="102" t="str">
+        <x:v>1. Elegir período: 1º bimestre, 1º cuatrimestre o 3º bimestre.</x:v>
+      </x:c>
+      <x:c r="B25" s="102" t="str"/>
+      <x:c r="C25" s="102" t="str"/>
+      <x:c r="D25" s="102" t="str"/>
+      <x:c r="E25" s="102" t="str">
+        <x:v>1º y 3º bimestre</x:v>
+      </x:c>
+      <x:c r="F25" s="102" t="str">
+        <x:v>En proceso; Suficiente; Avanzado; ACREDITÓ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="102" t="str">
+        <x:v>2. Elegir hoja origen: EPSI o EPSG.</x:v>
+      </x:c>
+      <x:c r="B26" s="102" t="str"/>
+      <x:c r="C26" s="102" t="str"/>
+      <x:c r="D26" s="102" t="str"/>
+      <x:c r="E26" s="102" t="str">
+        <x:v>1º cuatrimestre</x:v>
+      </x:c>
+      <x:c r="F26" s="102" t="str">
+        <x:v>Enteros 1 a 10; ACREDITÓ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="22" customHeight="1">
+      <x:c r="A27" s="102" t="str">
+        <x:v>3. Ingresar DNI y verificar las URL/ID de fuentes.</x:v>
+      </x:c>
+      <x:c r="B27" s="102" t="str"/>
+      <x:c r="C27" s="102" t="str"/>
+      <x:c r="D27" s="102" t="str"/>
+      <x:c r="E27" s="102" t="str">
+        <x:v>Excluidos</x:v>
+      </x:c>
+      <x:c r="F27" s="102" t="str">
+        <x:v>vacío; NO CURSA; CURSA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="22" customHeight="1">
+      <x:c r="A28" s="102" t="str">
+        <x:v>4. Ejecutar Informes EPS &gt; Generar informe actual.</x:v>
+      </x:c>
+      <x:c r="B28" s="102" t="str"/>
+      <x:c r="C28" s="102" t="str"/>
+      <x:c r="D28" s="102" t="str"/>
+      <x:c r="E28" s="102" t="str">
+        <x:v>No válidos 1º cuat.</x:v>
+      </x:c>
+      <x:c r="F28" s="102" t="str">
+        <x:v>decimales; texto junto con número; nota escrita como texto</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="22" customHeight="1">
+      <x:c r="A29" s="102" t="str">
+        <x:v>5. Revisar Informe_actual antes de imprimir o exportar.</x:v>
+      </x:c>
+      <x:c r="B29" s="102" t="str"/>
+      <x:c r="C29" s="102" t="str"/>
+      <x:c r="D29" s="102" t="str"/>
+      <x:c r="E29" s="102" t="str"/>
+      <x:c r="F29" s="102" t="str"/>
+    </x:row>
+    <x:row r="30" ht="22" customHeight="1">
+      <x:c r="A30" s="102" t="str"/>
+      <x:c r="B30" s="102" t="str"/>
+      <x:c r="C30" s="102" t="str"/>
+      <x:c r="D30" s="102" t="str"/>
+      <x:c r="E30" s="102" t="str"/>
+      <x:c r="F30" s="102" t="str"/>
+    </x:row>
+    <x:row r="31" ht="30" customHeight="1">
+      <x:c r="A31" s="82" t="str">
         <x:v>Reglas centrales</x:v>
       </x:c>
-      <x:c r="B21" s="82" t="str"/>
-      <x:c r="C21" s="82" t="str"/>
-      <x:c r="D21" s="82" t="str"/>
-      <x:c r="E21" s="82" t="str"/>
-      <x:c r="F21" s="82" t="str"/>
-    </x:row>
-    <x:row r="22" ht="30" customHeight="1">
-      <x:c r="A22" s="99" t="str">
+      <x:c r="B31" s="82" t="str"/>
+      <x:c r="C31" s="82" t="str"/>
+      <x:c r="D31" s="82" t="str"/>
+      <x:c r="E31" s="82" t="str"/>
+      <x:c r="F31" s="82" t="str"/>
+    </x:row>
+    <x:row r="32" ht="30" customHeight="1">
+      <x:c r="A32" s="99" t="str">
         <x:v>La hoja origen es la orientación del período a generar; en los períodos anteriores el DNI se busca en EPSI y EPSG.</x:v>
       </x:c>
-      <x:c r="B22" s="99" t="str"/>
-      <x:c r="C22" s="99" t="str"/>
-      <x:c r="D22" s="99" t="str"/>
-      <x:c r="E22" s="99" t="str"/>
-      <x:c r="F22" s="99" t="str"/>
-    </x:row>
-    <x:row r="23" ht="30" customHeight="1">
-      <x:c r="A23" s="99" t="str">
+      <x:c r="B32" s="99" t="str"/>
+      <x:c r="C32" s="99" t="str"/>
+      <x:c r="D32" s="99" t="str"/>
+      <x:c r="E32" s="99" t="str"/>
+      <x:c r="F32" s="99" t="str"/>
+    </x:row>
+    <x:row r="33" ht="30" customHeight="1">
+      <x:c r="A33" s="99" t="str">
         <x:v>Los informes de 1º cuatrimestre y 3º bimestre son acumulativos respecto de períodos anteriores. Para generar el 3º bimestre, pueden usarse fuentes de 1º bimestre y 1º cuatrimestre como antecedentes.</x:v>
       </x:c>
-      <x:c r="B23" s="99" t="str"/>
-      <x:c r="C23" s="99" t="str"/>
-      <x:c r="D23" s="99" t="str"/>
-      <x:c r="E23" s="99" t="str"/>
-      <x:c r="F23" s="99" t="str"/>
-    </x:row>
-    <x:row r="24" ht="30" customHeight="1">
-      <x:c r="A24" s="99" t="str">
+      <x:c r="B33" s="99" t="str"/>
+      <x:c r="C33" s="99" t="str"/>
+      <x:c r="D33" s="99" t="str"/>
+      <x:c r="E33" s="99" t="str"/>
+      <x:c r="F33" s="99" t="str"/>
+    </x:row>
+    <x:row r="34" ht="30" customHeight="1">
+      <x:c r="A34" s="99" t="str">
         <x:v>Las celdas de períodos sin calificación válida quedan vacías; no se completan con guion.</x:v>
       </x:c>
-      <x:c r="B24" s="99" t="str"/>
-      <x:c r="C24" s="99" t="str"/>
-      <x:c r="D24" s="99" t="str"/>
-      <x:c r="E24" s="99" t="str"/>
-      <x:c r="F24" s="99" t="str"/>
-    </x:row>
-    <x:row r="25" ht="30" customHeight="1">
-      <x:c r="A25" s="99" t="str">
+      <x:c r="B34" s="99" t="str"/>
+      <x:c r="C34" s="99" t="str"/>
+      <x:c r="D34" s="99" t="str"/>
+      <x:c r="E34" s="99" t="str"/>
+      <x:c r="F34" s="99" t="str"/>
+    </x:row>
+    <x:row r="35" ht="30" customHeight="1">
+      <x:c r="A35" s="99" t="str">
         <x:v>La información general sale siempre de la fuente principal del período generado.</x:v>
       </x:c>
-      <x:c r="B25" s="99" t="str"/>
-      <x:c r="C25" s="99" t="str"/>
-      <x:c r="D25" s="99" t="str"/>
-      <x:c r="E25" s="99" t="str"/>
-      <x:c r="F25" s="99" t="str"/>
+      <x:c r="B35" s="99" t="str"/>
+      <x:c r="C35" s="99" t="str"/>
+      <x:c r="D35" s="99" t="str"/>
+      <x:c r="E35" s="99" t="str"/>
+      <x:c r="F35" s="99" t="str"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="3">
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="B5">
       <x:formula1>"1º bimestre,1º cuatrimestre,3º bimestre"</x:formula1>
     </x:dataValidation>
@@ -15238,6 +15348,9 @@
     </x:dataValidation>
     <x:dataValidation type="list" sqref="B9">
       <x:formula1>"EPS1,EPS2,EPS3,EPS4"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="B15:B22">
+      <x:formula1>"SÍ,NO"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>